<commit_message>
Adopt held models across every importing script
Same cause as e2eTodaysFixes, eight more scripts: a fixture that invents its
own model names lands entirely HELD on the catalogue gate, and with no
unheld rows there is no "Load N rows" button — so the script dies waiting
for a control the app is right not to show, and records no checks at all.

adoptHeldModels walks the preview's own "Add to catalogue" affordance, which
is the documented flow, and is a no-op when nothing is held.

  e2eReportsInsightsBrutal              0 -> 22/22
  e2eSalesHistoryVoidedInclusionBrutal  0 ->   7/7
  e2eStockAlertsBrutal                  0 ->   6/6
  e2eSupplierAndBestSellersBrutal       0 -> 13/13

Suite total 660/683 -> 708/731.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/reports-insights-panels/fixtures/VELOCITY_INVENTORY.xlsx
+++ b/e2e-screenshots/reports-insights-panels/fixtures/VELOCITY_INVENTORY.xlsx
@@ -436,7 +436,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B2" t="str">
         <v>TESTBRAND VELOCITY FASTMOVER</v>
@@ -471,7 +471,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B3" t="str">
         <v>TESTBRAND VELOCITY FASTMOVER</v>
@@ -506,7 +506,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B4" t="str">
         <v>TESTBRAND VELOCITY FASTMOVER</v>
@@ -541,7 +541,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B5" t="str">
         <v>TESTBRAND VELOCITY FASTMOVER</v>
@@ -576,7 +576,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B6" t="str">
         <v>TESTBRAND VELOCITY FASTMOVER</v>
@@ -611,7 +611,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-07-17</v>
+        <v>2026-07-21</v>
       </c>
       <c r="B7" t="str">
         <v>TESTBRAND VELOCITY SLOWMOVER</v>
@@ -646,7 +646,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-07-17</v>
+        <v>2026-07-21</v>
       </c>
       <c r="B8" t="str">
         <v>TESTBRAND VELOCITY SLOWMOVER</v>
@@ -681,7 +681,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-07-17</v>
+        <v>2026-07-21</v>
       </c>
       <c r="B9" t="str">
         <v>TESTBRAND VELOCITY SLOWMOVER</v>
@@ -716,7 +716,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-07-17</v>
+        <v>2026-07-21</v>
       </c>
       <c r="B10" t="str">
         <v>TESTBRAND VELOCITY SLOWMOVER</v>
@@ -751,7 +751,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="B11" t="str">
         <v>TESTBRAND VELOCITY REORDERALERT</v>
@@ -786,7 +786,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="B12" t="str">
         <v>TESTBRAND VELOCITY REORDERALERT</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="B13" t="str">
         <v>TESTBRAND VELOCITY REORDERALERT</v>
@@ -856,7 +856,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="B14" t="str">
         <v>TESTBRAND VELOCITY REORDERALERT</v>
@@ -891,7 +891,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="B15" t="str">
         <v>TESTBRAND VELOCITY REORDERALERT</v>
@@ -926,7 +926,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="B16" t="str">
         <v>TESTBRAND VELOCITY REORDERALERT</v>

</xml_diff>